<commit_message>
REVIEW rebuilt with Shaw Road; handover for ChatGPT
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RKGFyarCMuMinKYL7AiBap
</commit_message>
<xml_diff>
--- a/FP/VP527277/Final/JCE_CostSheet_VP527277_RevH.xlsx
+++ b/FP/VP527277/Final/JCE_CostSheet_VP527277_RevH.xlsx
@@ -435,7 +435,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>JCE Infrastructure: VP527277 / MRC-2645 cost sheet Rev H (12/10/2026). JCE does vehicle road imaging and rating, drone capture and all GIS/register work in-house; no road imaging partner. Rates marked TBC are for Jayden to confirm.</t>
+          <t>JCE Infrastructure: VP527277 / MRC-2645 cost sheet Rev H, Our ref FP-022 (12/10/2026; rig $550/day cost basis, Year 1 capture/rating margin add-back $74,900 in the technician rate ($160 vs $110 cost basis) and capture day rate ($1,850 vs $550)). JCE does vehicle road imaging and rating, drone capture and all GIS/register work in-house; no road imaging partner. Rates marked TBC are for Jayden to confirm.</t>
         </is>
       </c>
     </row>
@@ -1611,11 +1611,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Daily remote QC of uploaded imagery (22 capture days)</t>
+          <t>Daily remote QC of uploaded imagery (about 27 capture days)</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Casual driver and field assistant: about 22 capture days, 3-day pilot, drone visual observer days, data offload and travel (fixed allowance) [TBC - Jayden]</t>
+          <t>Casual driver and field assistant: about 30 capture days including the pilot, contingency days, drone visual observer days, data offload and travel (fixed allowance, paid at or above award)</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
-        <v>10000</v>
+        <v>18000</v>
       </c>
       <c r="F43">
         <f>C43*E43</f>
@@ -1786,7 +1786,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Casual GIS and desktop rating technician: first-pass rating of about 300,000 road and roadside images and drone imagery, road defect coding, image processing, GIS layers, register population, image index, maps and report tables (718 h at $110/h charge rate; cost about $65/h)</t>
+          <t>Casual GIS and desktop rating technician: first-pass rating of about 300,000 road and roadside images and drone imagery, road defect coding, image processing, GIS layers, register population, image index, maps and report tables (718 h at the JCE CAD / GIS Technician rate of $160/h)</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1794,7 +1794,7 @@
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
-        <v>110</v>
+        <v>160</v>
       </c>
       <c r="F44">
         <f>C44*E44</f>
@@ -1835,14 +1835,14 @@
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Vehicle capture rig equipment rate (one 360/multi-camera system with GNSS/IMU and RTK, mounts, storage; covers lease or amortised purchase): 25 capture and pilot days at $350 per day [TBC - Jayden to confirm rate]</t>
+          <t>Vehicle capture day rate (Mosaic 51/X-class 360 rig with Emlid RS3 RTK GNSS, vehicle fit-out, data storage and image processing): 30 capture and pilot days at $1,850 per day</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
       <c r="F48" t="n">
-        <v>8750</v>
+        <v>55500</v>
       </c>
     </row>
     <row r="49">
@@ -1919,7 +1919,7 @@
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Rig backup: spare 360 camera and GNSS receiver, or short-term hire of a second rig if the first fails</t>
+          <t>Rig backup: budget 360 camera with RTK logger carried as a spare, or short-term hire of a second rig if capture falls more than a week behind</t>
         </is>
       </c>
       <c r="C54" t="inlineStr"/>
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>152180</v>
+        <v>156670</v>
       </c>
       <c r="D3">
         <f>C3*0.1</f>
@@ -2156,7 +2156,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>160420</v>
+        <v>165360</v>
       </c>
       <c r="D4">
         <f>C4*0.1</f>
@@ -2179,7 +2179,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>138200</v>
+        <v>140990</v>
       </c>
       <c r="D5">
         <f>C5*0.1</f>
@@ -2202,7 +2202,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>205330</v>
+        <v>210440</v>
       </c>
       <c r="D6">
         <f>C6*0.1</f>
@@ -2290,7 +2290,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>131030.6</v>
+        <v>154914.21</v>
       </c>
     </row>
     <row r="3">
@@ -2300,7 +2300,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>136342.64</v>
+        <v>161194.52</v>
       </c>
     </row>
     <row r="4">
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6925.34</v>
+        <v>8187.66</v>
       </c>
     </row>
     <row r="5">
@@ -2320,7 +2320,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17457.63</v>
+        <v>20639.72</v>
       </c>
     </row>
     <row r="6">
@@ -2330,7 +2330,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4898.89</v>
+        <v>5791.84</v>
       </c>
     </row>
     <row r="7">
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9915.83</v>
+        <v>11723.24</v>
       </c>
     </row>
     <row r="8">
@@ -2350,7 +2350,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>36712.17</v>
+        <v>43403.89</v>
       </c>
     </row>
     <row r="9">
@@ -2360,7 +2360,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16395.22</v>
+        <v>19383.66</v>
       </c>
     </row>
     <row r="10">
@@ -2370,7 +2370,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1377.2</v>
+        <v>1628.23</v>
       </c>
     </row>
     <row r="11">
@@ -2380,7 +2380,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>129063.16</v>
+        <v>152588.18</v>
       </c>
     </row>
     <row r="12">
@@ -2390,7 +2390,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>9181.32</v>
+        <v>10854.85</v>
       </c>
     </row>
     <row r="13">
@@ -2492,7 +2492,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C4" t="n">
         <v>4</v>
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C5" t="n">
         <v>4.4</v>

</xml_diff>